<commit_message>
fix: finalize demo auth and data hygiene
</commit_message>
<xml_diff>
--- a/docs/demo-import/学生导入_203班_演示.xlsx
+++ b/docs/demo-import/学生导入_203班_演示.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学生导入" sheetId="1" r:id="R22198e70abcf4ff9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="R05e57d290d1b41de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="学生导入" sheetId="1" r:id="Rf73fa33587214ef1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="2" r:id="Rc1a6a589e47f4027"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -396,10 +396,10 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>S20360001</x:v>
+        <x:v>2026203004</x:v>
       </x:c>
       <x:c r="B2" s="2" t="str">
-        <x:v>林知远</x:v>
+        <x:v>顾清扬</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
         <x:v>CLASS_203</x:v>
@@ -408,33 +408,23 @@
         <x:v>高三</x:v>
       </x:c>
       <x:c r="E2" s="2" t="str">
-        <x:v>s203_demo_lin</x:v>
+        <x:v>2026203004</x:v>
       </x:c>
-      <x:c r="F2" s="2" t="str"/>
+      <x:c r="F2" s="2" t="str">
+        <x:v>a1234567</x:v>
+      </x:c>
       <x:c r="G2" s="2" t="str">
         <x:v>ENABLED</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="2" t="str">
-        <x:v>S20360002</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="str">
-        <x:v>沈思宁</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="str">
-        <x:v>CLASS_203</x:v>
-      </x:c>
-      <x:c r="D3" s="2" t="str">
-        <x:v>高三</x:v>
-      </x:c>
-      <x:c r="E3" s="2" t="str">
-        <x:v>s203_demo_shen</x:v>
-      </x:c>
-      <x:c r="F3" s="2" t="str"/>
-      <x:c r="G3" s="2" t="str">
-        <x:v>ENABLED</x:v>
-      </x:c>
+      <x:c r="A3" s="2"/>
+      <x:c r="B3" s="2"/>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+      <x:c r="G3" s="2"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="n"/>

</xml_diff>